<commit_message>
java array, java instanse+실습문제
</commit_message>
<xml_diff>
--- a/A00_index.xlsx
+++ b/A00_index.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lect\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\lecture\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0151B2-6936-4FB2-91EF-0F00F284B52F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82DB5F46-AB6F-4069-AFB5-25C1A5F7C8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -19,17 +19,26 @@
     <sheet name="C02_javascript" sheetId="3" r:id="rId4"/>
     <sheet name="C04_java" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="59">
   <si>
     <t>C00_html</t>
   </si>
@@ -117,6 +126,126 @@
   </si>
   <si>
     <t>C:\lect\C00_html\html900_영역\html902_시맨틱태그_영역_인라인블록_ver001+250709.html</t>
+  </si>
+  <si>
+    <t>section05</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Application</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Application2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Application3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Application5</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Application4</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>dementional</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>배열 예시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>배열예시</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2차원 배열</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>chap05</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>copy</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>얕은 복사</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>얕은복사 활용</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>깊은 복사</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>깊은복사 활용</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>sort</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정렬</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>section06</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>클래스</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Member</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>클래스를 쓰는 이유</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Monster</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">직접접근 </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>문제2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>문제1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>문제3</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>section02 encaptsulation</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">Monster 필드 변수의 이름을 변경시 main method를 다 바꿔야한다. </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>직접 접근은 private로 막고 public 메소드 getter setter를 사용</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -629,9 +758,177 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE5F1543-67CE-4086-B440-1841205D1B1D}">
-  <dimension ref="A1"/>
+  <dimension ref="E2:I21"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
-  <sheetData/>
+  <cols>
+    <col min="5" max="5" width="11.59765625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E6" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="9" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H9" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="10" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="H10" t="s">
+        <v>30</v>
+      </c>
+      <c r="I10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E11" t="s">
+        <v>35</v>
+      </c>
+      <c r="H11" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E12" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H12" t="s">
+        <v>53</v>
+      </c>
+      <c r="I12" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="H13" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E14" t="s">
+        <v>40</v>
+      </c>
+      <c r="H14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="15" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E15" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" t="s">
+        <v>55</v>
+      </c>
+      <c r="I15" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="5:9" x14ac:dyDescent="0.4">
+      <c r="E16" t="s">
+        <v>31</v>
+      </c>
+      <c r="F16" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="5:8" x14ac:dyDescent="0.4">
+      <c r="E17" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" t="s">
+        <v>43</v>
+      </c>
+      <c r="H17" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="5:8" x14ac:dyDescent="0.4">
+      <c r="E18" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="5:8" x14ac:dyDescent="0.4">
+      <c r="E20" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="21" spans="5:8" x14ac:dyDescent="0.4">
+      <c r="E21" t="s">
+        <v>30</v>
+      </c>
+      <c r="F21" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>